<commit_message>
Update ESP32-S3 BOM spreadsheet for component tracking
</commit_message>
<xml_diff>
--- a/Hexapod/ESP32-S3_BOM.xlsx
+++ b/Hexapod/ESP32-S3_BOM.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hexapod\Hexapod\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B5D82D-5143-4C59-8293-308B5B20F1C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,12 +24,84 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
+  </si>
+  <si>
+    <t>Part Number</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>ESP32-s3</t>
+  </si>
+  <si>
+    <t>Current sensor</t>
+  </si>
+  <si>
+    <t>Mouser No: 356-ESP32S3MINI1UN8</t>
+  </si>
+  <si>
+    <t>ESP32-S3-MINI-1U-N8</t>
+  </si>
+  <si>
+    <t>Espressif Systems</t>
+  </si>
+  <si>
+    <t>INA260AIPWR</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t>Mouser No: 595-INA260AIPWR</t>
+  </si>
+  <si>
+    <t>IMU</t>
+  </si>
+  <si>
+    <t>Mouser No: 262-BMI330</t>
+  </si>
+  <si>
+    <t>BMI330</t>
+  </si>
+  <si>
+    <t>Bosch Sensortec</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -37,7 +115,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,14 +123,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +421,91 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="22.85546875" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" customWidth="1"/>
+    <col min="4" max="4" width="27" customWidth="1"/>
+    <col min="5" max="5" width="81.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{3C0D68C1-D269-4ABC-ACB7-8B4F9738844C}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{53848EB4-BDCF-4B24-8975-E6603DDE0EEB}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{7CEA2E71-D25B-4D2E-915D-1AD4A457C43F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added items to BOM
</commit_message>
<xml_diff>
--- a/Hexapod/ESP32-S3_BOM.xlsx
+++ b/Hexapod/ESP32-S3_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hexapod\Hexapod\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Raven\Documents\Hexapod\Hexapod\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9949B5-9DBA-4B28-8101-75311D3FEDAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70675BB2-CCB8-4B23-811C-157FF39F6E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>Quantity</t>
   </si>
@@ -76,6 +76,36 @@
   </si>
   <si>
     <t>Bosch Sensortec</t>
+  </si>
+  <si>
+    <t>Battery Monitor</t>
+  </si>
+  <si>
+    <t>Mouser No: 595-BQ7692006PWR</t>
+  </si>
+  <si>
+    <t>BQ7692006PWR</t>
+  </si>
+  <si>
+    <t>Battery Charger</t>
+  </si>
+  <si>
+    <t>BQ24610RGER</t>
+  </si>
+  <si>
+    <t>Mouser No: 595-BQ24610RGER</t>
+  </si>
+  <si>
+    <t>Mouser No: 584-LTM4620AEV#PBF</t>
+  </si>
+  <si>
+    <t>LTM4620AEV#PBF</t>
+  </si>
+  <si>
+    <t>5V regulator IC</t>
+  </si>
+  <si>
+    <t>Analog Devices</t>
   </si>
 </sst>
 </file>
@@ -422,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.85546875" customWidth="1"/>
@@ -499,13 +529,67 @@
         <v>14</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{3C0D68C1-D269-4ABC-ACB7-8B4F9738844C}"/>
     <hyperlink ref="E3" r:id="rId2" xr:uid="{53848EB4-BDCF-4B24-8975-E6603DDE0EEB}"/>
     <hyperlink ref="E4" r:id="rId3" xr:uid="{7CEA2E71-D25B-4D2E-915D-1AD4A457C43F}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{C6698D0E-5549-4F7E-B764-648BC9F0D34D}"/>
+    <hyperlink ref="E6" r:id="rId5" xr:uid="{D7F6E889-80FF-421A-B93C-FB4CB07C565F}"/>
+    <hyperlink ref="E7" r:id="rId6" xr:uid="{C5374C56-F962-40C8-A763-FFC726787BD6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>